<commit_message>
alterada a celula A5
</commit_message>
<xml_diff>
--- a/pipeline/templates/Graficos auxiliares.xlsx
+++ b/pipeline/templates/Graficos auxiliares.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\dashboard\alonissos\AAAAAA_novissimo\alonissos-api\pipeline\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26A4F8C-F9C7-4046-95DD-7657B69D4742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9896CA9E-51D2-4F19-99D7-9871735625F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{87F32D68-C7BE-44F3-B84C-3143EB0CF62A}"/>
   </bookViews>
@@ -2398,9 +2398,9 @@
       </c>
     </row>
     <row r="2" spans="1:56">
-      <c r="A2">
-        <f>I8</f>
-        <v>0</v>
+      <c r="A2" t="str">
+        <f>escolha_do_sku!A5</f>
+        <v>A</v>
       </c>
       <c r="B2" t="str">
         <f>escolha_do_sku!B5</f>

</xml_diff>